<commit_message>
ng: update the nigeria forms
</commit_message>
<xml_diff>
--- a/ONCHO/Entomological survey Survey/Nigeria/2025/ng_oncho_2503_1_community_tar.xlsx
+++ b/ONCHO/Entomological survey Survey/Nigeria/2025/ng_oncho_2503_1_community_tar.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yumbad\Repositories\dsa-forms\ONCHO\Entomological survey Survey\Nigeria\2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FA0A8A2-7AED-4A23-9BC8-0B4A15EC0B78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0FAC8DD-4BE4-4916-9AFD-C3AA640350EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="survey" sheetId="1" r:id="rId1"/>
@@ -245,9 +245,6 @@
     <t>ng_oncho_2503_1_community_tar</t>
   </si>
   <si>
-    <t>(Taraba) 1. Community Registration Form</t>
-  </si>
-  <si>
     <t>TARABA</t>
   </si>
   <si>
@@ -639,6 +636,9 @@
   </si>
   <si>
     <t/>
+  </si>
+  <si>
+    <t>(Taraba) 1. Community Registration Form V4</t>
   </si>
 </sst>
 </file>
@@ -1614,10 +1614,10 @@
         <v>56</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -1625,13 +1625,13 @@
         <v>57</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -1639,13 +1639,13 @@
         <v>57</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D9" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -1653,13 +1653,13 @@
         <v>57</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D10" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -1667,13 +1667,13 @@
         <v>57</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -1681,13 +1681,13 @@
         <v>57</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D12" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -1695,13 +1695,13 @@
         <v>57</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D13" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -1709,13 +1709,13 @@
         <v>57</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D14" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -1723,13 +1723,13 @@
         <v>57</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -1737,13 +1737,13 @@
         <v>57</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D16" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -1751,13 +1751,13 @@
         <v>57</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D17" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -1765,13 +1765,13 @@
         <v>57</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D18" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -1779,13 +1779,13 @@
         <v>57</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D19" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
@@ -1793,13 +1793,13 @@
         <v>57</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D20" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -1807,13 +1807,13 @@
         <v>57</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D21" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -1824,13 +1824,13 @@
         <v>62</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E23" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
@@ -1838,13 +1838,13 @@
         <v>62</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E24" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
@@ -1852,13 +1852,13 @@
         <v>62</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E25" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
@@ -1866,13 +1866,13 @@
         <v>62</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E26" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
@@ -1880,13 +1880,13 @@
         <v>62</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E27" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
@@ -1894,13 +1894,13 @@
         <v>62</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E28" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
@@ -1908,13 +1908,13 @@
         <v>62</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E29" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
@@ -1922,13 +1922,13 @@
         <v>62</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E30" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
@@ -1936,13 +1936,13 @@
         <v>62</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E31" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
@@ -1950,13 +1950,13 @@
         <v>62</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E32" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
@@ -1964,13 +1964,13 @@
         <v>62</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E33" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
@@ -1978,13 +1978,13 @@
         <v>62</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E34" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
@@ -1992,13 +1992,13 @@
         <v>62</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E35" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
@@ -2006,13 +2006,13 @@
         <v>62</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E36" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
@@ -2020,13 +2020,13 @@
         <v>62</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E37" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
@@ -2034,13 +2034,13 @@
         <v>62</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E38" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
@@ -2048,13 +2048,13 @@
         <v>62</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E39" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
@@ -2062,13 +2062,13 @@
         <v>62</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E40" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
@@ -2076,13 +2076,13 @@
         <v>62</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E41" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
@@ -2090,13 +2090,13 @@
         <v>62</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E42" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
@@ -2104,13 +2104,13 @@
         <v>62</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E43" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
@@ -2118,13 +2118,13 @@
         <v>62</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E44" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
@@ -2132,13 +2132,13 @@
         <v>62</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E45" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
@@ -2146,13 +2146,13 @@
         <v>62</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E46" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
@@ -2160,13 +2160,13 @@
         <v>62</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E47" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
@@ -2174,13 +2174,13 @@
         <v>62</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E48" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="49" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
@@ -2188,13 +2188,13 @@
         <v>62</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E49" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
@@ -2202,13 +2202,13 @@
         <v>62</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E50" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
@@ -2216,13 +2216,13 @@
         <v>62</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E51" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
@@ -2230,13 +2230,13 @@
         <v>62</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E52" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
@@ -2244,13 +2244,13 @@
         <v>62</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E53" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
@@ -2258,13 +2258,13 @@
         <v>62</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E54" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
@@ -2272,13 +2272,13 @@
         <v>62</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E55" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
@@ -2286,13 +2286,13 @@
         <v>62</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E56" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
@@ -2300,13 +2300,13 @@
         <v>62</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E57" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
@@ -2314,13 +2314,13 @@
         <v>62</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E58" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
@@ -2328,13 +2328,13 @@
         <v>62</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E59" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
@@ -2342,13 +2342,13 @@
         <v>62</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E60" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
@@ -2356,13 +2356,13 @@
         <v>62</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E61" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
@@ -2370,13 +2370,13 @@
         <v>62</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E62" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
@@ -2384,13 +2384,13 @@
         <v>62</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E63" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
@@ -2398,13 +2398,13 @@
         <v>62</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E64" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
@@ -2412,13 +2412,13 @@
         <v>62</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E65" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
@@ -2426,13 +2426,13 @@
         <v>62</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E66" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
@@ -2440,13 +2440,13 @@
         <v>62</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E67" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
@@ -2454,13 +2454,13 @@
         <v>62</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E68" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
@@ -2468,13 +2468,13 @@
         <v>62</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E69" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
@@ -2482,13 +2482,13 @@
         <v>62</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E70" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
@@ -2496,13 +2496,13 @@
         <v>62</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E71" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
@@ -2510,13 +2510,13 @@
         <v>62</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E72" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
@@ -2524,13 +2524,13 @@
         <v>62</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E73" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
@@ -2538,13 +2538,13 @@
         <v>62</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E74" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
@@ -2552,13 +2552,13 @@
         <v>62</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E75" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
@@ -2566,13 +2566,13 @@
         <v>62</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E76" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
@@ -2580,13 +2580,13 @@
         <v>62</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E77" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
@@ -2594,13 +2594,13 @@
         <v>62</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E78" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
@@ -2608,13 +2608,13 @@
         <v>62</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E79" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
@@ -2622,13 +2622,13 @@
         <v>62</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E80" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
@@ -2636,13 +2636,13 @@
         <v>67</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F82" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
@@ -2650,13 +2650,13 @@
         <v>67</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F83" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
@@ -2664,13 +2664,13 @@
         <v>67</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F84" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
@@ -2678,13 +2678,13 @@
         <v>67</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F85" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
@@ -2692,13 +2692,13 @@
         <v>67</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F86" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
@@ -2706,13 +2706,13 @@
         <v>67</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F87" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
@@ -2720,13 +2720,13 @@
         <v>67</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F88" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
@@ -2734,13 +2734,13 @@
         <v>67</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F89" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
@@ -2748,13 +2748,13 @@
         <v>67</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="F90" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.25">
@@ -2762,13 +2762,13 @@
         <v>67</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="F91" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
@@ -2776,13 +2776,13 @@
         <v>67</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C92" s="1" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F92" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
@@ -2790,13 +2790,13 @@
         <v>67</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="F93" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
@@ -2804,13 +2804,13 @@
         <v>67</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C94" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F94" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.25">
@@ -2818,13 +2818,13 @@
         <v>67</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F95" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.25">
@@ -2832,13 +2832,13 @@
         <v>67</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F96" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
@@ -2846,13 +2846,13 @@
         <v>67</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F97" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
@@ -2860,13 +2860,13 @@
         <v>67</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C98" s="1" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="F98" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.25">
@@ -2874,13 +2874,13 @@
         <v>67</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C99" s="1" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F99" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.25">
@@ -2888,13 +2888,13 @@
         <v>67</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F100" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
@@ -2902,13 +2902,13 @@
         <v>67</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F101" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.25">
@@ -2916,13 +2916,13 @@
         <v>67</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C102" s="1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F102" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.25">
@@ -2930,13 +2930,13 @@
         <v>67</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C103" s="1" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F103" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.25">
@@ -2944,13 +2944,13 @@
         <v>67</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C104" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F104" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.25">
@@ -2958,13 +2958,13 @@
         <v>67</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C105" s="1" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F105" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.25">
@@ -2972,13 +2972,13 @@
         <v>67</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C106" s="1" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F106" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.25">
@@ -2986,13 +2986,13 @@
         <v>67</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C107" s="1" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F107" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.25">
@@ -3000,13 +3000,13 @@
         <v>67</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C108" s="1" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F108" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.25">
@@ -3014,13 +3014,13 @@
         <v>67</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C109" s="1" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F109" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.25">
@@ -3028,13 +3028,13 @@
         <v>67</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C110" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F110" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.25">
@@ -3042,13 +3042,13 @@
         <v>67</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C111" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F111" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.25">
@@ -3056,13 +3056,13 @@
         <v>67</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C112" s="1" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F112" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.25">
@@ -3070,13 +3070,13 @@
         <v>67</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C113" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F113" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.25">
@@ -3084,13 +3084,13 @@
         <v>67</v>
       </c>
       <c r="B114" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C114" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F114" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.25">
@@ -3098,13 +3098,13 @@
         <v>67</v>
       </c>
       <c r="B115" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C115" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F115" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.25">
@@ -3112,13 +3112,13 @@
         <v>67</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C116" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F116" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.25">
@@ -3126,13 +3126,13 @@
         <v>67</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C117" s="1" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F117" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.25">
@@ -3140,13 +3140,13 @@
         <v>67</v>
       </c>
       <c r="B118" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C118" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F118" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.25">
@@ -3154,13 +3154,13 @@
         <v>67</v>
       </c>
       <c r="B119" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C119" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F119" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.25">
@@ -3168,13 +3168,13 @@
         <v>67</v>
       </c>
       <c r="B120" s="1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C120" s="1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F120" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.25">
@@ -3182,13 +3182,13 @@
         <v>67</v>
       </c>
       <c r="B121" s="1" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C121" s="1" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F121" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.25">
@@ -3196,13 +3196,13 @@
         <v>67</v>
       </c>
       <c r="B122" s="1" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C122" s="1" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F122" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.25">
@@ -3210,13 +3210,13 @@
         <v>67</v>
       </c>
       <c r="B123" s="1" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C123" s="1" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F123" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.25">
@@ -3224,13 +3224,13 @@
         <v>67</v>
       </c>
       <c r="B124" s="1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C124" s="1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F124" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.25">
@@ -3238,13 +3238,13 @@
         <v>67</v>
       </c>
       <c r="B125" s="1" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C125" s="1" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F125" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.25">
@@ -3252,13 +3252,13 @@
         <v>67</v>
       </c>
       <c r="B126" s="1" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C126" s="1" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F126" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.25">
@@ -3266,13 +3266,13 @@
         <v>67</v>
       </c>
       <c r="B127" s="1" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C127" s="1" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F127" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.25">
@@ -3280,13 +3280,13 @@
         <v>67</v>
       </c>
       <c r="B128" s="1" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C128" s="1" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="F128" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.25">
@@ -3294,13 +3294,13 @@
         <v>67</v>
       </c>
       <c r="B129" s="1" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C129" s="1" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F129" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.25">
@@ -3308,13 +3308,13 @@
         <v>67</v>
       </c>
       <c r="B130" s="1" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C130" s="1" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F130" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.25">
@@ -3322,13 +3322,13 @@
         <v>67</v>
       </c>
       <c r="B131" s="1" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C131" s="1" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F131" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.25">
@@ -3336,13 +3336,13 @@
         <v>67</v>
       </c>
       <c r="B132" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C132" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F132" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.25">
@@ -3350,13 +3350,13 @@
         <v>67</v>
       </c>
       <c r="B133" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C133" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F133" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.25">
@@ -3364,13 +3364,13 @@
         <v>67</v>
       </c>
       <c r="B134" s="1" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C134" s="1" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F134" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.25">
@@ -3378,13 +3378,13 @@
         <v>67</v>
       </c>
       <c r="B135" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C135" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="F135" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.25">
@@ -3392,13 +3392,13 @@
         <v>67</v>
       </c>
       <c r="B136" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C136" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F136" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.25">
@@ -3406,13 +3406,13 @@
         <v>67</v>
       </c>
       <c r="B137" s="1" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C137" s="1" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F137" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="138" spans="1:6" x14ac:dyDescent="0.25">
@@ -3420,13 +3420,13 @@
         <v>67</v>
       </c>
       <c r="B138" s="1" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C138" s="1" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F138" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.25">
@@ -3434,23 +3434,23 @@
         <v>67</v>
       </c>
       <c r="B139" s="1" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C139" s="1" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="F139" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.25">
       <c r="F140" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.25">
       <c r="F141" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
   </sheetData>
@@ -3486,7 +3486,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>69</v>
+        <v>200</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>68</v>

</xml_diff>